<commit_message>
fix: la Responsable garde un droit de refus apres validation du comite
</commit_message>
<xml_diff>
--- a/backend/docs/dictionnaire_donnees_mmf.xlsx
+++ b/backend/docs/dictionnaire_donnees_mmf.xlsx
@@ -2760,7 +2760,7 @@
       <c r="E81" s="3" t="inlineStr"/>
       <c r="F81" s="3" t="inlineStr">
         <is>
-          <t>EnCours, Validee, Rejetee — recalculé à partir des 3 Validation liées</t>
+          <t>EnCours, EnAttenteResponsable (comité a valide en interne, en attente de decision de la Responsable), Validee, Rejetee</t>
         </is>
       </c>
     </row>
@@ -3830,7 +3830,7 @@
       </c>
       <c r="D118" s="3" t="inlineStr">
         <is>
-          <t>NOT NULL</t>
+          <t>NULL</t>
         </is>
       </c>
       <c r="E118" s="3" t="inlineStr">
@@ -3840,7 +3840,7 @@
       </c>
       <c r="F118" s="3" t="inlineStr">
         <is>
-          <t>Le membre du comité qui a traité cette étape précise</t>
+          <t>Qui a traité cette étape — NULL tant que l'étape est en attente, rempli au moment du traitement (approbation/rejet)</t>
         </is>
       </c>
     </row>

</xml_diff>